<commit_message>
Fixed feed rations and slaughter ages and weights in the steers scenario
</commit_message>
<xml_diff>
--- a/scenarios/steers.xlsx
+++ b/scenarios/steers.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="31">
   <si>
     <t>parameter</t>
   </si>
@@ -34,16 +34,134 @@
   </si>
   <si>
     <t>y_0</t>
+  </si>
+  <si>
+    <t>dairy</t>
+  </si>
+  <si>
+    <t>steers</t>
+  </si>
+  <si>
+    <t>share_in_ration</t>
+  </si>
+  <si>
+    <t>ley silage, regrowth</t>
+  </si>
+  <si>
+    <t>grazing</t>
+  </si>
+  <si>
+    <t>orig.</t>
+  </si>
+  <si>
+    <t>new</t>
+  </si>
+  <si>
+    <t>beef</t>
+  </si>
+  <si>
+    <t>f_breed</t>
+  </si>
+  <si>
+    <t>f_animal</t>
+  </si>
+  <si>
+    <t>f_feed</t>
+  </si>
+  <si>
+    <t>Feed rations</t>
+  </si>
+  <si>
+    <t>Share castrated</t>
+  </si>
+  <si>
+    <t>slaughter_age</t>
+  </si>
+  <si>
+    <t>months</t>
+  </si>
+  <si>
+    <t>Slaughter age</t>
+  </si>
+  <si>
+    <t>%</t>
+  </si>
+  <si>
+    <t>rel</t>
+  </si>
+  <si>
+    <t>other feeds changed proportionally</t>
+  </si>
+  <si>
+    <t>varies by breed and prod_system</t>
+  </si>
+  <si>
+    <t>Slaughter and live weight</t>
+  </si>
+  <si>
+    <t>slaughter_weight</t>
+  </si>
+  <si>
+    <t>kg CW</t>
+  </si>
+  <si>
+    <t>live_weight_slaughter</t>
+  </si>
+  <si>
+    <t>changes proportionally to slaughter weight</t>
+  </si>
+  <si>
+    <t>kg</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="1" x14ac:knownFonts="1">
+  <numFmts count="1">
+    <numFmt numFmtId="168" formatCode="0.0"/>
+  </numFmts>
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <u/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="2" tint="-0.249977111117893"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="4"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -69,8 +187,17 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="168" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="168" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -351,37 +478,409 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C2"/>
+  <dimension ref="A1:K22"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="30.5703125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="6" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="7" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="18.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="30.5703125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="6" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="7" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="E1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="F1" s="1" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
+      <c r="H1" t="s">
+        <v>10</v>
+      </c>
+      <c r="I1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A2" s="2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="D3" t="s">
         <v>3</v>
       </c>
-      <c r="B2" t="s">
+      <c r="E3" t="s">
         <v>2</v>
       </c>
-      <c r="C2">
+      <c r="F3" s="5">
+        <f>I3</f>
         <v>100</v>
+      </c>
+      <c r="H3" t="s">
+        <v>24</v>
+      </c>
+      <c r="I3" s="8">
+        <v>100</v>
+      </c>
+      <c r="J3" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A5" s="2" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>5</v>
+      </c>
+      <c r="B6" t="s">
+        <v>6</v>
+      </c>
+      <c r="D6" t="s">
+        <v>18</v>
+      </c>
+      <c r="E6" t="s">
+        <v>2</v>
+      </c>
+      <c r="F6" s="3">
+        <f>I6</f>
+        <v>29.050688450113576</v>
+      </c>
+      <c r="H6" s="3">
+        <v>29.050688450113576</v>
+      </c>
+      <c r="I6" s="6">
+        <f>H6</f>
+        <v>29.050688450113576</v>
+      </c>
+      <c r="J6" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>12</v>
+      </c>
+      <c r="B7" t="s">
+        <v>6</v>
+      </c>
+      <c r="D7" t="s">
+        <v>18</v>
+      </c>
+      <c r="E7" t="s">
+        <v>2</v>
+      </c>
+      <c r="F7" s="3">
+        <f>I7</f>
+        <v>30</v>
+      </c>
+      <c r="H7" s="3">
+        <v>27.558030529284888</v>
+      </c>
+      <c r="I7" s="8">
+        <v>30</v>
+      </c>
+      <c r="J7" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="E8" s="3"/>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A9" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="E9" s="3"/>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>5</v>
+      </c>
+      <c r="B10" t="s">
+        <v>6</v>
+      </c>
+      <c r="D10" t="s">
+        <v>26</v>
+      </c>
+      <c r="E10" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="F10" s="3">
+        <f>I10</f>
+        <v>328.06056613664163</v>
+      </c>
+      <c r="H10" s="3">
+        <v>328.06056613664163</v>
+      </c>
+      <c r="I10" s="6">
+        <f>H10</f>
+        <v>328.06056613664163</v>
+      </c>
+      <c r="J10" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>12</v>
+      </c>
+      <c r="B11" t="s">
+        <v>6</v>
+      </c>
+      <c r="D11" t="s">
+        <v>26</v>
+      </c>
+      <c r="E11" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="F11" s="3">
+        <f>I11</f>
+        <v>385</v>
+      </c>
+      <c r="H11" s="3">
+        <v>335.97588628947517</v>
+      </c>
+      <c r="I11" s="9">
+        <v>385</v>
+      </c>
+      <c r="J11" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>5</v>
+      </c>
+      <c r="B12" t="s">
+        <v>6</v>
+      </c>
+      <c r="D12" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="E12" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="F12" s="4">
+        <f>I10/H10</f>
+        <v>1</v>
+      </c>
+      <c r="H12" s="3">
+        <v>640.74329323562813</v>
+      </c>
+      <c r="I12" s="6">
+        <f>H12*F12</f>
+        <v>640.74329323562813</v>
+      </c>
+      <c r="J12" t="s">
+        <v>30</v>
+      </c>
+      <c r="K12" s="3" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>12</v>
+      </c>
+      <c r="B13" t="s">
+        <v>6</v>
+      </c>
+      <c r="D13" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="E13" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="F13" s="4">
+        <f>I11/H11</f>
+        <v>1.145915572251176</v>
+      </c>
+      <c r="H13" s="3">
+        <v>631.22742272568064</v>
+      </c>
+      <c r="I13" s="6">
+        <f>H13*F13</f>
+        <v>723.33333333333337</v>
+      </c>
+      <c r="J13" t="s">
+        <v>30</v>
+      </c>
+      <c r="K13" s="3" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A15" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>5</v>
+      </c>
+      <c r="B16" t="s">
+        <v>6</v>
+      </c>
+      <c r="C16" t="s">
+        <v>8</v>
+      </c>
+      <c r="D16" t="s">
+        <v>7</v>
+      </c>
+      <c r="E16" t="s">
+        <v>2</v>
+      </c>
+      <c r="F16">
+        <f>H16</f>
+        <v>55.029062371648976</v>
+      </c>
+      <c r="H16" s="3">
+        <v>55.029062371648976</v>
+      </c>
+      <c r="I16" s="6">
+        <f>H16</f>
+        <v>55.029062371648976</v>
+      </c>
+      <c r="J16" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="17" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>5</v>
+      </c>
+      <c r="B17" t="s">
+        <v>6</v>
+      </c>
+      <c r="C17" t="s">
+        <v>9</v>
+      </c>
+      <c r="D17" t="s">
+        <v>7</v>
+      </c>
+      <c r="E17" t="s">
+        <v>2</v>
+      </c>
+      <c r="F17">
+        <f>H17</f>
+        <v>38.614788214420173</v>
+      </c>
+      <c r="H17" s="3">
+        <v>38.614788214420173</v>
+      </c>
+      <c r="I17" s="6">
+        <f>H17</f>
+        <v>38.614788214420173</v>
+      </c>
+      <c r="J17" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="18" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>5</v>
+      </c>
+      <c r="B18" t="s">
+        <v>6</v>
+      </c>
+      <c r="D18" t="s">
+        <v>7</v>
+      </c>
+      <c r="E18" t="s">
+        <v>22</v>
+      </c>
+      <c r="F18" s="4">
+        <f>(1/(100-SUM(H16:H17))*(1-SUM(I16:I17)/100)*100)</f>
+        <v>1.0000000000000007</v>
+      </c>
+      <c r="H18" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="20" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>12</v>
+      </c>
+      <c r="B20" t="s">
+        <v>6</v>
+      </c>
+      <c r="C20" t="s">
+        <v>8</v>
+      </c>
+      <c r="D20" t="s">
+        <v>7</v>
+      </c>
+      <c r="E20" t="s">
+        <v>2</v>
+      </c>
+      <c r="H20" s="3">
+        <v>69.016974351370379</v>
+      </c>
+      <c r="I20" s="9">
+        <f>100*0.53685</f>
+        <v>53.685000000000002</v>
+      </c>
+      <c r="J20" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="21" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>12</v>
+      </c>
+      <c r="B21" t="s">
+        <v>6</v>
+      </c>
+      <c r="C21" t="s">
+        <v>9</v>
+      </c>
+      <c r="D21" t="s">
+        <v>7</v>
+      </c>
+      <c r="E21" t="s">
+        <v>2</v>
+      </c>
+      <c r="H21" s="3">
+        <v>30.282083494235561</v>
+      </c>
+      <c r="I21" s="9">
+        <f>0.4574*100</f>
+        <v>45.739999999999995</v>
+      </c>
+      <c r="J21" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="22" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="E22" t="s">
+        <v>22</v>
+      </c>
+      <c r="F22" s="4">
+        <f>(1/(100-SUM(H20:H21))*(1-SUM(I20:I21)/100)*100)</f>
+        <v>0.82032446813970517</v>
+      </c>
+      <c r="H22" t="s">
+        <v>23</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>